<commit_message>
Companion site update for the JIDM revision: noWorkflow 2.1.1 graphs, prompts, analysis, multiscript package
</commit_message>
<xml_diff>
--- a/mappings.xlsx
+++ b/mappings.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet state="visible" name="Nodes" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Edges" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Analysis" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Analysis_2018" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Analysis" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -5189,7 +5190,7 @@
         <v>13</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>14</v>
@@ -10911,4 +10912,533 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="13" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analysis: values reported in the revised paper (2026). Computed by the scripts in analysis/ on the graphs in output/provenance; the complete outputs (trails, matched nodes and edges) are in analysis/results/. The sheet Analysis_2018 keeps the original computation over the graphs of the first submission and is superseded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table 3 (Section 4.6.2): functional and variable components</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|AI|</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP_func AI-&gt;G</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FP_func</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP_func G-&gt;AI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FN_func</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|G|</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP_var</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FP_var</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FN_var (incl. 7 ports)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SP</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SR</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monolithic</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0.0</v>
+      </c>
+      <c r="D5">
+        <v>0.0</v>
+      </c>
+      <c r="E5">
+        <v>0.0</v>
+      </c>
+      <c r="F5">
+        <v>14.0</v>
+      </c>
+      <c r="G5">
+        <v>14</v>
+      </c>
+      <c r="H5">
+        <v>16</v>
+      </c>
+      <c r="I5">
+        <v>861</v>
+      </c>
+      <c r="J5">
+        <v>31</v>
+      </c>
+      <c r="K5">
+        <v>0.018</v>
+      </c>
+      <c r="L5">
+        <v>0.262</v>
+      </c>
+      <c r="M5">
+        <v>0.034</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expert-modularized</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>14.0</v>
+      </c>
+      <c r="D6">
+        <v>0.0</v>
+      </c>
+      <c r="E6">
+        <v>14.0</v>
+      </c>
+      <c r="F6">
+        <v>0.0</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>40</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>0.982</v>
+      </c>
+      <c r="L6">
+        <v>0.885</v>
+      </c>
+      <c r="M6">
+        <v>0.931</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LLM-modularized (Gemini)</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>6.83</v>
+      </c>
+      <c r="D7">
+        <v>1.17</v>
+      </c>
+      <c r="E7">
+        <v>9.43</v>
+      </c>
+      <c r="F7">
+        <v>4.57</v>
+      </c>
+      <c r="G7">
+        <v>14</v>
+      </c>
+      <c r="H7">
+        <v>31</v>
+      </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7">
+        <v>16</v>
+      </c>
+      <c r="K7">
+        <v>0.841</v>
+      </c>
+      <c r="L7">
+        <v>0.663</v>
+      </c>
+      <c r="M7">
+        <v>0.741</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 8 (Section 4.6.1): monolithic graph, exact matching over all nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FP</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FN</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recall</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-Measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monolithic</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>1343</v>
+      </c>
+      <c r="D11">
+        <v>45</v>
+      </c>
+      <c r="E11">
+        <v>0.012</v>
+      </c>
+      <c r="F11">
+        <v>0.262</v>
+      </c>
+      <c r="G11">
+        <v>0.023</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge comparison (Section 4.6.1): one-to-one, orientation ignored; sheet Edges with row 10 corrected</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ground-truth edges</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Candidate graph edges</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FN</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FP</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recall</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-Measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expert-modularized</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>95</v>
+      </c>
+      <c r="C15">
+        <v>93</v>
+      </c>
+      <c r="D15">
+        <v>89</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+      <c r="F15">
+        <v>4</v>
+      </c>
+      <c r="G15">
+        <v>0.957</v>
+      </c>
+      <c r="H15">
+        <v>0.937</v>
+      </c>
+      <c r="I15">
+        <v>0.947</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monolithic</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>95</v>
+      </c>
+      <c r="C16">
+        <v>63</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>95</v>
+      </c>
+      <c r="F16">
+        <v>63</v>
+      </c>
+      <c r="G16">
+        <v>0.0</v>
+      </c>
+      <c r="H16">
+        <v>0.0</v>
+      </c>
+      <c r="I16">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Robustness check (Section 9): top-level variables matched by name and final value, no ports</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FP</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FN</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SP</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SR</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monolithic</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>22</v>
+      </c>
+      <c r="C20">
+        <v>56</v>
+      </c>
+      <c r="D20">
+        <v>15</v>
+      </c>
+      <c r="E20">
+        <v>0.282</v>
+      </c>
+      <c r="F20">
+        <v>0.431</v>
+      </c>
+      <c r="G20">
+        <v>0.341</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LLM-modularized (Gemini)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21">
+        <v>14</v>
+      </c>
+      <c r="D21">
+        <v>17</v>
+      </c>
+      <c r="E21">
+        <v>0.639</v>
+      </c>
+      <c r="F21">
+        <v>0.577</v>
+      </c>
+      <c r="G21">
+        <v>0.606</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expert-modularized (self-comparison)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>37</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>1.0</v>
+      </c>
+      <c r="F22">
+        <v>1.0</v>
+      </c>
+      <c r="G22">
+        <v>1.0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>